<commit_message>
feat(bulk-ui): add upload format guide and sample file downloads (.txt, .csv, .xlsx)
- Clarify upload format: 1 comment per line, no header required
- Add direct sample file download endpoints and UI buttons for .txt, .csv, .xlsx
- Enhance bulk parser in bulk_processor.py to support headerless files without losing row 1
- Include pre-formatted sample_car_comments.csv with UTF-8-SIG encoding
</commit_message>
<xml_diff>
--- a/demo_flask/sample_car_comments.xlsx
+++ b/demo_flask/sample_car_comments.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,116 +413,109 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>comment</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Xe chạy rất êm ái, cách âm vượt trội so với các đối thủ cùng phân khúc</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Xe chạy rất êm ái, cách âm vượt trội so với các đối thủ cùng phân khúc</t>
+          <t>Chạy được 3 tháng đã lỗi pin, đại lý bảo hành thiếu trách nhiệm quá thất vọng</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Chạy được 3 tháng đã lỗi pin, đại lý bảo hành thiếu trách nhiệm quá thất vọng</t>
+          <t>Tiện cho mình xin phép hỏi chi phí lăn bánh tại Hà Nội và thủ tục trả góp với ạ?</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tiện cho mình xin phép hỏi chi phí lăn bánh tại Hà Nội và thủ tục trả góp với ạ?</t>
+          <t>Tầm tiền này chọn VF3 là quá hợp lý cho chị em đi phố che mưa nắng</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tầm tiền này chọn VF3 là quá hợp lý cho chị em đi phố che mưa nắng</t>
+          <t>Điều hòa mát sâu, cách âm tốt nhưng phần mềm màn hình thỉnh thoảng còn đơ nhẹ</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Điều hòa mát sâu, cách âm tốt nhưng phần mềm màn hình thỉnh thoảng còn đơ nhẹ</t>
+          <t>Xe đi rung lắc khi lên dải tốc độ 100km/h trên cao tốc, cảm giác không an toàn</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Xe đi rung lắc khi lên dải tốc độ 100km/h trên cao tốc, cảm giác không an toàn</t>
+          <t>Chính sách miễn phí sạc pin của hãng đợt này rất được lòng cộng đồng người dùng</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Chính sách miễn phí sạc pin của hãng đợt này rất được lòng cộng đồng người dùng</t>
+          <t>Đang tính mua mà lăn tăn vụ thiếu trạm sạc ở các huyện vùng sâu quá mọi người ơi</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Đang tính mua mà lăn tăn vụ thiếu trạm sạc ở các huyện vùng sâu quá mọi người ơi</t>
+          <t>Hệ thống phanh ABS và cân bằng điện tử hoạt động nhạy, cảm biến lùi rất chuẩn xác</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Hệ thống phanh ABS và cân bằng điện tử hoạt động nhạy, cảm biến lùi rất chuẩn xác</t>
+          <t>Dịch vụ cứu hộ pin 24/7 đến chậm hơn 2 tiếng đồng hồ làm lỡ hết công việc của khách</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dịch vụ cứu hộ pin 24/7 đến chậm hơn 2 tiếng đồng hồ làm lỡ hết công việc của khách</t>
+          <t>550tr lăn bánh còn thừa cầm về, gầm cao 5 chỗ mới tinh lh: 0918.079.865</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>550tr lăn bánh còn thừa cầm về, gầm cao 5 chỗ mới tinh lh: 0918.079.865</t>
+          <t>Chi phí vận hành và bảo dưỡng xe điện tiết kiệm hơn xe xăng rất nhiều</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Chi phí vận hành và bảo dưỡng xe điện tiết kiệm hơn xe xăng rất nhiều</t>
+          <t>Màu sơn thực tế bên ngoài nhìn bóng bẩy và sang hơn trong hình chụp quảng cáo</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Màu sơn thực tế bên ngoài nhìn bóng bẩy và sang hơn trong hình chụp quảng cáo</t>
+          <t>Cốp sau hơi khiêm tốn nếu gia đình đi du lịch dài ngày mang nhiều vali</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
-        <is>
-          <t>Cốp sau hơi khiêm tốn nếu gia đình đi du lịch dài ngày mang nhiều vali</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
         <is>
           <t>Đã lái thử 2 lần và quyết định cọc luôn bản Plus, trải nghiệm lái vượt tầm giá tiền</t>
         </is>

</xml_diff>